<commit_message>
Sjednotit intervaly kapitoly 2 na horni mez vcetne
</commit_message>
<xml_diff>
--- a/data/kapitola_02.xlsx
+++ b/data/kapitola_02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R Projects\github\statistics-for-psychology\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE3B78C2-BDC9-4873-8BE4-3EB60FCCD27A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67FB27E0-9D80-461F-A6A0-B6398ED30607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4184" yWindow="2771" windowWidth="25839" windowHeight="16071" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cetnosti" sheetId="1" r:id="rId1"/>
@@ -106,27 +106,6 @@
     <t>Interval (h)</t>
   </si>
   <si>
-    <t>4 až &lt; 5</t>
-  </si>
-  <si>
-    <t>5 až &lt; 6</t>
-  </si>
-  <si>
-    <t>6 až &lt; 7</t>
-  </si>
-  <si>
-    <t>7 až &lt; 8</t>
-  </si>
-  <si>
-    <t>8 až &lt; 9</t>
-  </si>
-  <si>
-    <t>9 až &lt; 10</t>
-  </si>
-  <si>
-    <t>Dolní mez patří do intervalu, horní už ne. Intervaly mají šířku 1 hodina.</t>
-  </si>
-  <si>
     <t>Tři z 36 účastníků spánek neuvedli. Prázdná buňka neznamená 0 hodin.</t>
   </si>
   <si>
@@ -296,6 +275,27 @@
   </si>
   <si>
     <t>P36</t>
+  </si>
+  <si>
+    <t>&gt; 4 až 5</t>
+  </si>
+  <si>
+    <t>&gt; 5 až 6</t>
+  </si>
+  <si>
+    <t>&gt; 6 až 7</t>
+  </si>
+  <si>
+    <t>&gt; 7 až 8</t>
+  </si>
+  <si>
+    <t>&gt; 8 až 9</t>
+  </si>
+  <si>
+    <t>&gt; 9 až 10</t>
+  </si>
+  <si>
+    <t>Dolní mez nepatří do intervalu, horní ano. Intervaly mají šířku 1 hodina.</t>
   </si>
 </sst>
 </file>
@@ -741,22 +741,22 @@
               <c:strCache>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>4 až &lt; 5</c:v>
+                  <c:v>&gt; 4 až 5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5 až &lt; 6</c:v>
+                  <c:v>&gt; 5 až 6</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6 až &lt; 7</c:v>
+                  <c:v>&gt; 6 až 7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>7 až &lt; 8</c:v>
+                  <c:v>&gt; 7 až 8</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8 až &lt; 9</c:v>
+                  <c:v>&gt; 8 až 9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>9 až &lt; 10</c:v>
+                  <c:v>&gt; 9 až 10</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -768,22 +768,22 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2239,19 +2239,19 @@
         <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="D5" s="6">
-        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;="&amp;A5,Data!$B$2:$B$37,"&lt;"&amp;B5)</f>
-        <v>2</v>
+        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A5,Data!$B$2:$B$37,"&lt;="&amp;B5)</f>
+        <v>3</v>
       </c>
       <c r="E5" s="7">
         <f t="shared" ref="E5:E10" si="0">D5/$C$2</f>
-        <v>6.0606060606060608E-2</v>
+        <v>9.0909090909090912E-2</v>
       </c>
       <c r="F5" s="8">
         <f t="shared" ref="F5:F10" si="1">E5</f>
-        <v>6.0606060606060608E-2</v>
+        <v>9.0909090909090912E-2</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -2273,19 +2273,19 @@
         <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D6" s="6">
-        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;="&amp;A6,Data!$B$2:$B$37,"&lt;"&amp;B6)</f>
-        <v>4</v>
+        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A6,Data!$B$2:$B$37,"&lt;="&amp;B6)</f>
+        <v>5</v>
       </c>
       <c r="E6" s="7">
         <f t="shared" si="0"/>
-        <v>0.12121212121212122</v>
+        <v>0.15151515151515152</v>
       </c>
       <c r="F6" s="8">
         <f t="shared" si="1"/>
-        <v>0.12121212121212122</v>
+        <v>0.15151515151515152</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
@@ -2307,19 +2307,19 @@
         <v>7</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>25</v>
+        <v>82</v>
       </c>
       <c r="D7" s="6">
-        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;="&amp;A7,Data!$B$2:$B$37,"&lt;"&amp;B7)</f>
-        <v>7</v>
+        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A7,Data!$B$2:$B$37,"&lt;="&amp;B7)</f>
+        <v>8</v>
       </c>
       <c r="E7" s="7">
         <f t="shared" si="0"/>
-        <v>0.21212121212121213</v>
+        <v>0.24242424242424243</v>
       </c>
       <c r="F7" s="8">
         <f t="shared" si="1"/>
-        <v>0.21212121212121213</v>
+        <v>0.24242424242424243</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -2341,19 +2341,19 @@
         <v>8</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="D8" s="6">
-        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;="&amp;A8,Data!$B$2:$B$37,"&lt;"&amp;B8)</f>
-        <v>11</v>
+        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A8,Data!$B$2:$B$37,"&lt;="&amp;B8)</f>
+        <v>10</v>
       </c>
       <c r="E8" s="7">
         <f t="shared" si="0"/>
-        <v>0.33333333333333331</v>
+        <v>0.30303030303030304</v>
       </c>
       <c r="F8" s="8">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
+        <v>0.30303030303030304</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -2375,19 +2375,19 @@
         <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="D9" s="6">
-        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;="&amp;A9,Data!$B$2:$B$37,"&lt;"&amp;B9)</f>
-        <v>6</v>
+        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A9,Data!$B$2:$B$37,"&lt;="&amp;B9)</f>
+        <v>5</v>
       </c>
       <c r="E9" s="7">
         <f t="shared" si="0"/>
-        <v>0.18181818181818182</v>
+        <v>0.15151515151515152</v>
       </c>
       <c r="F9" s="8">
         <f t="shared" si="1"/>
-        <v>0.18181818181818182</v>
+        <v>0.15151515151515152</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
@@ -2409,19 +2409,19 @@
         <v>10</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>28</v>
+        <v>85</v>
       </c>
       <c r="D10" s="6">
-        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;="&amp;A10,Data!$B$2:$B$37,"&lt;"&amp;B10)</f>
-        <v>3</v>
+        <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A10,Data!$B$2:$B$37,"&lt;="&amp;B10)</f>
+        <v>2</v>
       </c>
       <c r="E10" s="7">
         <f t="shared" si="0"/>
-        <v>9.0909090909090912E-2</v>
+        <v>6.0606060606060608E-2</v>
       </c>
       <c r="F10" s="8">
         <f t="shared" si="1"/>
-        <v>9.0909090909090912E-2</v>
+        <v>6.0606060606060608E-2</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -2505,7 +2505,7 @@
     </row>
     <row r="14" spans="1:17" ht="22.1" customHeight="1">
       <c r="A14" s="12" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -2526,7 +2526,7 @@
     </row>
     <row r="15" spans="1:17" ht="22.1" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2566,7 +2566,7 @@
     </row>
     <row r="17" spans="1:17" ht="22.1" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -2587,7 +2587,7 @@
     </row>
     <row r="18" spans="1:17" ht="22.1" customHeight="1">
       <c r="A18" s="12" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -3042,23 +3042,23 @@
   <sheetData>
     <row r="1" spans="1:17" ht="36" customHeight="1">
       <c r="A1" s="3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -3073,7 +3073,7 @@
     </row>
     <row r="2" spans="1:17" ht="22.1" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B2" s="13">
         <v>6</v>
@@ -3082,7 +3082,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E2" s="14">
         <v>2</v>
@@ -3102,7 +3102,7 @@
     </row>
     <row r="3" spans="1:17" ht="22.1" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B3" s="13">
         <v>8</v>
@@ -3111,14 +3111,14 @@
         <v>9</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E3" s="14">
         <v>4</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="12" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -3133,7 +3133,7 @@
     </row>
     <row r="4" spans="1:17" ht="22.1" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="B4" s="13">
         <v>7</v>
@@ -3142,14 +3142,14 @@
         <v>8</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E4" s="14">
         <v>3</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="12" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -3164,7 +3164,7 @@
     </row>
     <row r="5" spans="1:17" ht="22.1" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="B5" s="13">
         <v>5</v>
@@ -3173,14 +3173,14 @@
         <v>6</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E5" s="14">
         <v>2</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="12" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -3195,21 +3195,21 @@
     </row>
     <row r="6" spans="1:17" ht="22.1" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B6" s="13"/>
       <c r="C6" s="14">
         <v>7</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E6" s="14">
         <v>3</v>
       </c>
       <c r="F6" s="1"/>
       <c r="G6" s="12" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -3224,7 +3224,7 @@
     </row>
     <row r="7" spans="1:17" ht="22.1" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="B7" s="13">
         <v>7</v>
@@ -3233,14 +3233,14 @@
         <v>0</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E7" s="14">
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
       <c r="G7" s="12" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -3255,7 +3255,7 @@
     </row>
     <row r="8" spans="1:17" ht="22.1" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B8" s="13">
         <v>4.5</v>
@@ -3264,14 +3264,14 @@
         <v>2</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E8" s="14">
         <v>1</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="12" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -3286,7 +3286,7 @@
     </row>
     <row r="9" spans="1:17" ht="22.1" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="B9" s="13">
         <v>6.3</v>
@@ -3295,14 +3295,14 @@
         <v>7</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E9" s="14">
         <v>3</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="12" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -3317,7 +3317,7 @@
     </row>
     <row r="10" spans="1:17" ht="22.1" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="B10" s="13">
         <v>7.3</v>
@@ -3326,14 +3326,14 @@
         <v>9</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E10" s="14">
         <v>4</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="12" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -3348,7 +3348,7 @@
     </row>
     <row r="11" spans="1:17" ht="22.1" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="B11" s="13">
         <v>8.1</v>
@@ -3357,14 +3357,14 @@
         <v>4</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E11" s="14">
         <v>2</v>
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="12" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -3379,21 +3379,21 @@
     </row>
     <row r="12" spans="1:17" ht="22.1" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="B12" s="13"/>
       <c r="C12" s="14">
         <v>7</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E12" s="14">
         <v>3</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="12" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -3408,7 +3408,7 @@
     </row>
     <row r="13" spans="1:17" ht="22.1" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="B13" s="13">
         <v>6</v>
@@ -3417,7 +3417,7 @@
         <v>10</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E13" s="14">
         <v>2</v>
@@ -3437,7 +3437,7 @@
     </row>
     <row r="14" spans="1:17" ht="22.1" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="B14" s="13">
         <v>7.1</v>
@@ -3446,7 +3446,7 @@
         <v>5</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E14" s="14">
         <v>3</v>
@@ -3466,7 +3466,7 @@
     </row>
     <row r="15" spans="1:17" ht="22.1" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B15" s="13">
         <v>7.9</v>
@@ -3475,7 +3475,7 @@
         <v>8</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E15" s="14">
         <v>1</v>
@@ -3495,7 +3495,7 @@
     </row>
     <row r="16" spans="1:17" ht="22.1" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="B16" s="13">
         <v>9.1999999999999993</v>
@@ -3504,7 +3504,7 @@
         <v>11</v>
       </c>
       <c r="D16" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E16" s="14">
         <v>3</v>
@@ -3524,7 +3524,7 @@
     </row>
     <row r="17" spans="1:17" ht="22.1" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B17" s="13">
         <v>5.5</v>
@@ -3533,7 +3533,7 @@
         <v>6</v>
       </c>
       <c r="D17" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E17" s="14">
         <v>4</v>
@@ -3553,7 +3553,7 @@
     </row>
     <row r="18" spans="1:17" ht="22.1" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B18" s="13">
         <v>6.8</v>
@@ -3562,7 +3562,7 @@
         <v>8</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E18" s="14">
         <v>2</v>
@@ -3582,7 +3582,7 @@
     </row>
     <row r="19" spans="1:17" ht="22.1" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B19" s="13">
         <v>7.5</v>
@@ -3591,7 +3591,7 @@
         <v>3</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E19" s="14">
         <v>4</v>
@@ -3611,7 +3611,7 @@
     </row>
     <row r="20" spans="1:17" ht="22.1" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="B20" s="13">
         <v>8.8000000000000007</v>
@@ -3620,7 +3620,7 @@
         <v>7</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E20" s="14">
         <v>2</v>
@@ -3640,7 +3640,7 @@
     </row>
     <row r="21" spans="1:17" ht="22.1" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="B21" s="13">
         <v>4.8</v>
@@ -3649,7 +3649,7 @@
         <v>9</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E21" s="14">
         <v>3</v>
@@ -3669,7 +3669,7 @@
     </row>
     <row r="22" spans="1:17" ht="22.1" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="B22" s="13">
         <v>6.5</v>
@@ -3678,7 +3678,7 @@
         <v>5</v>
       </c>
       <c r="D22" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E22" s="14">
         <v>1</v>
@@ -3698,7 +3698,7 @@
     </row>
     <row r="23" spans="1:17" ht="22.1" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B23" s="13">
         <v>7.4</v>
@@ -3707,7 +3707,7 @@
         <v>7</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E23" s="14">
         <v>3</v>
@@ -3727,7 +3727,7 @@
     </row>
     <row r="24" spans="1:17" ht="22.1" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B24" s="13">
         <v>8.3000000000000007</v>
@@ -3736,7 +3736,7 @@
         <v>10</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E24" s="14">
         <v>4</v>
@@ -3756,14 +3756,14 @@
     </row>
     <row r="25" spans="1:17" ht="22.1" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="B25" s="13"/>
       <c r="C25" s="14">
         <v>6</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E25" s="14">
         <v>3</v>
@@ -3783,7 +3783,7 @@
     </row>
     <row r="26" spans="1:17" ht="22.1" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="B26" s="13">
         <v>6.2</v>
@@ -3792,7 +3792,7 @@
         <v>8</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E26" s="14">
         <v>4</v>
@@ -3812,7 +3812,7 @@
     </row>
     <row r="27" spans="1:17" ht="22.1" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="B27" s="13">
         <v>7.2</v>
@@ -3821,7 +3821,7 @@
         <v>12</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E27" s="14">
         <v>2</v>
@@ -3841,7 +3841,7 @@
     </row>
     <row r="28" spans="1:17" ht="22.1" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B28" s="13">
         <v>8</v>
@@ -3850,7 +3850,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E28" s="14">
         <v>3</v>
@@ -3870,7 +3870,7 @@
     </row>
     <row r="29" spans="1:17" ht="22.1" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B29" s="13">
         <v>9.5</v>
@@ -3879,7 +3879,7 @@
         <v>9</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E29" s="14">
         <v>2</v>
@@ -3899,7 +3899,7 @@
     </row>
     <row r="30" spans="1:17" ht="22.1" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B30" s="13">
         <v>5.8</v>
@@ -3908,7 +3908,7 @@
         <v>4</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E30" s="14">
         <v>3</v>
@@ -3928,7 +3928,7 @@
     </row>
     <row r="31" spans="1:17" ht="22.1" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B31" s="13">
         <v>7</v>
@@ -3937,7 +3937,7 @@
         <v>7</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E31" s="14">
         <v>4</v>
@@ -3957,7 +3957,7 @@
     </row>
     <row r="32" spans="1:17" ht="22.1" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B32" s="13">
         <v>7.7</v>
@@ -3966,7 +3966,7 @@
         <v>10</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E32" s="14">
         <v>3</v>
@@ -3986,7 +3986,7 @@
     </row>
     <row r="33" spans="1:17" ht="22.1" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B33" s="13">
         <v>9</v>
@@ -3995,7 +3995,7 @@
         <v>5</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E33" s="14">
         <v>4</v>
@@ -4015,7 +4015,7 @@
     </row>
     <row r="34" spans="1:17" ht="22.1" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B34" s="13">
         <v>5.2</v>
@@ -4024,7 +4024,7 @@
         <v>8</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E34" s="14">
         <v>2</v>
@@ -4044,7 +4044,7 @@
     </row>
     <row r="35" spans="1:17" ht="22.1" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B35" s="13">
         <v>6.5</v>
@@ -4053,7 +4053,7 @@
         <v>11</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E35" s="14">
         <v>3</v>
@@ -4073,7 +4073,7 @@
     </row>
     <row r="36" spans="1:17" ht="22.1" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B36" s="13">
         <v>7.5</v>
@@ -4082,7 +4082,7 @@
         <v>6</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E36" s="14">
         <v>2</v>
@@ -4102,7 +4102,7 @@
     </row>
     <row r="37" spans="1:17" ht="22.1" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B37" s="13">
         <v>8.5</v>
@@ -4111,7 +4111,7 @@
         <v>8</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E37" s="14">
         <v>3</v>

</xml_diff>

<commit_message>
Sjednotit data kapitol 1–4 do excelových sešitů
</commit_message>
<xml_diff>
--- a/data/kapitola_02.xlsx
+++ b/data/kapitola_02.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\R Projects\github\statistics-for-psychology\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67FB27E0-9D80-461F-A6A0-B6398ED30607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B73AE155-EF1B-484F-92CF-6DF8C0697109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Cetnosti" sheetId="1" r:id="rId1"/>
-    <sheet name="Histogram" sheetId="2" r:id="rId2"/>
-    <sheet name="Data" sheetId="3" r:id="rId3"/>
+    <sheet name="Prehled" sheetId="1" r:id="rId1"/>
+    <sheet name="Cetnosti" sheetId="2" r:id="rId2"/>
+    <sheet name="Histogram" sheetId="3" r:id="rId3"/>
+    <sheet name="Data" sheetId="4" r:id="rId4"/>
+    <sheet name="Sest_osob" sheetId="5" r:id="rId5"/>
+    <sheet name="Strategie" sheetId="6" r:id="rId6"/>
+    <sheet name="Tvary" sheetId="7" r:id="rId7"/>
+    <sheet name="Podlaha_strop" sheetId="8" r:id="rId8"/>
+    <sheet name="Stonek" sheetId="9" r:id="rId9"/>
+    <sheet name="U01_odpocatost" sheetId="10" r:id="rId10"/>
+    <sheet name="U03_chybeni" sheetId="11" r:id="rId11"/>
+    <sheet name="U03_ruseni" sheetId="12" r:id="rId12"/>
+    <sheet name="U04_chyby" sheetId="13" r:id="rId13"/>
+    <sheet name="U05_spanek" sheetId="14" r:id="rId14"/>
+    <sheet name="U08_stonek" sheetId="15" r:id="rId15"/>
+    <sheet name="Podpora" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +48,157 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="179">
+  <si>
+    <t>Data ke kapitole 2</t>
+  </si>
+  <si>
+    <t>Začněte vstupy. Žluté buňky obsahují data; modré buňky na výpočtových listech vzorce.</t>
+  </si>
+  <si>
+    <t>Zadání a vysvětlení jsou v kapitole. Řešení otevírejte až po vlastním pokusu.</t>
+  </si>
+  <si>
+    <t>Slovní úlohy bez konkrétních pozorování nevyžadují vlastní datový list.</t>
+  </si>
+  <si>
+    <t>Hladké modelové křivky jsou modely, nikoli další soubory naměřených hodnot.</t>
+  </si>
+  <si>
+    <t>List</t>
+  </si>
+  <si>
+    <t>Oblast vstupů / tabulky</t>
+  </si>
+  <si>
+    <t>Příklad nebo cvičení</t>
+  </si>
+  <si>
+    <t>Sest_osob</t>
+  </si>
+  <si>
+    <t>A2:E7</t>
+  </si>
+  <si>
+    <t>Úvodní příklad, jmenovatel procent</t>
+  </si>
+  <si>
+    <t>Strategie</t>
+  </si>
+  <si>
+    <t>A2:B4</t>
+  </si>
+  <si>
+    <t>Výsečový a sloupcový graf</t>
+  </si>
+  <si>
+    <t>Tvary</t>
+  </si>
+  <si>
+    <t>A2:G10</t>
+  </si>
+  <si>
+    <t>Obrázek: šest tvarů rozdělení</t>
+  </si>
+  <si>
+    <t>Podlaha_strop</t>
+  </si>
+  <si>
+    <t>A2:C14</t>
+  </si>
+  <si>
+    <t>Obrázek: meze nástroje</t>
+  </si>
+  <si>
+    <t>Stonek</t>
+  </si>
+  <si>
+    <t>A2:A9</t>
+  </si>
+  <si>
+    <t>Výklad: stonek a list</t>
+  </si>
+  <si>
+    <t>U01_odpocatost</t>
+  </si>
+  <si>
+    <t>A2:A13</t>
+  </si>
+  <si>
+    <t>Cvičení 1 a 2</t>
+  </si>
+  <si>
+    <t>U03_chybeni</t>
+  </si>
+  <si>
+    <t>Cvičení 3a</t>
+  </si>
+  <si>
+    <t>U03_ruseni</t>
+  </si>
+  <si>
+    <t>A2:C4</t>
+  </si>
+  <si>
+    <t>Cvičení 3b</t>
+  </si>
+  <si>
+    <t>U04_chyby</t>
+  </si>
+  <si>
+    <t>A2:A11</t>
+  </si>
+  <si>
+    <t>Cvičení 4</t>
+  </si>
+  <si>
+    <t>U05_spanek</t>
+  </si>
+  <si>
+    <t>Cvičení 5</t>
+  </si>
+  <si>
+    <t>U08_stonek</t>
+  </si>
+  <si>
+    <t>Cvičení 8: zadání k rekonstrukci</t>
+  </si>
+  <si>
+    <t>Podpora</t>
+  </si>
+  <si>
+    <t>A2:C3</t>
+  </si>
+  <si>
+    <t>Zavádějící graf; cvičení 9</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>A2:E37</t>
+  </si>
+  <si>
+    <t>36 osob; výklad a cvičení 10</t>
+  </si>
+  <si>
+    <t>Cetnosti</t>
+  </si>
+  <si>
+    <t>A4:H8</t>
+  </si>
+  <si>
+    <t>Hotové výpočty a graf odpočatosti</t>
+  </si>
+  <si>
+    <t>Histogram</t>
+  </si>
+  <si>
+    <t>A4:E10</t>
+  </si>
+  <si>
+    <t>Hotové intervalové četnosti a histogram</t>
+  </si>
   <si>
     <t>Odpočatost před úlohou</t>
   </si>
@@ -106,6 +269,27 @@
     <t>Interval (h)</t>
   </si>
   <si>
+    <t>&gt; 4 až 5</t>
+  </si>
+  <si>
+    <t>&gt; 5 až 6</t>
+  </si>
+  <si>
+    <t>&gt; 6 až 7</t>
+  </si>
+  <si>
+    <t>&gt; 7 až 8</t>
+  </si>
+  <si>
+    <t>&gt; 8 až 9</t>
+  </si>
+  <si>
+    <t>&gt; 9 až 10</t>
+  </si>
+  <si>
+    <t>Dolní mez nepatří do intervalu, horní ano. Intervaly mají šířku 1 hodina.</t>
+  </si>
+  <si>
     <t>Tři z 36 účastníků spánek neuvedli. Prázdná buňka neznamená 0 hodin.</t>
   </si>
   <si>
@@ -277,25 +461,130 @@
     <t>P36</t>
   </si>
   <si>
-    <t>&gt; 4 až 5</t>
-  </si>
-  <si>
-    <t>&gt; 5 až 6</t>
-  </si>
-  <si>
-    <t>&gt; 6 až 7</t>
-  </si>
-  <si>
-    <t>&gt; 7 až 8</t>
-  </si>
-  <si>
-    <t>&gt; 8 až 9</t>
-  </si>
-  <si>
-    <t>&gt; 9 až 10</t>
-  </si>
-  <si>
-    <t>Dolní mez nepatří do intervalu, horní ano. Intervaly mají šířku 1 hodina.</t>
+    <t>Použití a původ</t>
+  </si>
+  <si>
+    <t>Autorské ilustrační údaje. Nejde o skutečný výzkum.</t>
+  </si>
+  <si>
+    <t>Procvičování</t>
+  </si>
+  <si>
+    <t>Čtení</t>
+  </si>
+  <si>
+    <t>Vysvětlování</t>
+  </si>
+  <si>
+    <t>Hodnota</t>
+  </si>
+  <si>
+    <t>Souměrnost</t>
+  </si>
+  <si>
+    <t>Šikmost doprava</t>
+  </si>
+  <si>
+    <t>Šikmost doleva</t>
+  </si>
+  <si>
+    <t>Dva vrcholy</t>
+  </si>
+  <si>
+    <t>Rovnoměrnost</t>
+  </si>
+  <si>
+    <t>Odlehlost</t>
+  </si>
+  <si>
+    <t>Autorské schematické četnosti. Sloupce představují šest různých rozdělení, nikoli spárovaná měření lidí.</t>
+  </si>
+  <si>
+    <t>Počet správných odpovědí</t>
+  </si>
+  <si>
+    <t>Podlaha: četnost</t>
+  </si>
+  <si>
+    <t>Strop: četnost</t>
+  </si>
+  <si>
+    <t>Doba (s)</t>
+  </si>
+  <si>
+    <t>Odpočatost (kód 1–4)</t>
+  </si>
+  <si>
+    <t>Autorské údaje. 1 vůbec, 2 trochu, 3 dost, 4 zcela.</t>
+  </si>
+  <si>
+    <t>Odpověď</t>
+  </si>
+  <si>
+    <t>Ano</t>
+  </si>
+  <si>
+    <t>Ne</t>
+  </si>
+  <si>
+    <t>Chybí</t>
+  </si>
+  <si>
+    <t>Zadáno 25 oslovených; 20 odpovědělo. Četnosti, nikoli jednotliví lidé.</t>
+  </si>
+  <si>
+    <t>Možnost</t>
+  </si>
+  <si>
+    <t>Počet označení</t>
+  </si>
+  <si>
+    <t>Počet odpovídajících</t>
+  </si>
+  <si>
+    <t>Hluk</t>
+  </si>
+  <si>
+    <t>Telefon</t>
+  </si>
+  <si>
+    <t>Únava</t>
+  </si>
+  <si>
+    <t>Bylo možné označit více možností. Překryvy mezi lidmi nejsou zadány.</t>
+  </si>
+  <si>
+    <t>Počet chyb</t>
+  </si>
+  <si>
+    <t>Spánek (h)</t>
+  </si>
+  <si>
+    <t>Intervaly: více než 4 až 5 včetně, více než 5 až 6 včetně, více než 6 až 7 včetně, více než 7 až 8 včetně.</t>
+  </si>
+  <si>
+    <t>Listy</t>
+  </si>
+  <si>
+    <t>1 3 3 8</t>
+  </si>
+  <si>
+    <t>0 5</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Klíč: 2 | 3 znamená 23 sekund. Sloupec Listy je záměrně textový zápis zadání, nikoli hotové řešení.</t>
+  </si>
+  <si>
+    <t>Skupina</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
   </si>
 </sst>
 </file>
@@ -307,7 +596,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -343,10 +632,21 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF526775"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF223744"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -368,6 +668,11 @@
         <fgColor rgb="FFFFF8E7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF1CB"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -380,15 +685,21 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -426,6 +737,21 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -458,7 +784,7 @@
           <a:lstStyle/>
           <a:p>
             <a:r>
-              <a:rPr lang="cs-CZ" sz="1125">
+              <a:rPr sz="1125">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -488,7 +814,7 @@
               <a:srgbClr val="267888"/>
             </a:solidFill>
           </c:spPr>
-          <c:invertIfNegative val="1"/>
+          <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
               <c:f>Cetnosti!$B$5:$B$8</c:f>
@@ -531,17 +857,8 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
-              <c14:invertSolidFillFmt>
-                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </c14:spPr>
-              </c14:invertSolidFillFmt>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-5B12-4AE9-AE0A-8CE683D2AECB}"/>
+              <c16:uniqueId val="{00000000-D822-41B8-9D4B-67F4E0AE0A1D}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -581,7 +898,6 @@
               <a:lstStyle/>
               <a:p>
                 <a:r>
-                  <a:rPr lang="cs-CZ"/>
                   <a:t>Odpočatost</a:t>
                 </a:r>
               </a:p>
@@ -639,7 +955,6 @@
               <a:lstStyle/>
               <a:p>
                 <a:r>
-                  <a:rPr lang="cs-CZ"/>
                   <a:t>Počet účastníků</a:t>
                 </a:r>
               </a:p>
@@ -734,7 +1049,7 @@
               <a:srgbClr val="267888"/>
             </a:solidFill>
           </c:spPr>
-          <c:invertIfNegative val="1"/>
+          <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
               <c:f>Histogram!$C$5:$C$10</c:f>
@@ -789,17 +1104,8 @@
             </c:numRef>
           </c:val>
           <c:extLst>
-            <c:ext xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" uri="{6F2FDCE9-48DA-4B69-8628-5D25D57E5C99}">
-              <c14:invertSolidFillFmt>
-                <c14:spPr xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart">
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF"/>
-                  </a:solidFill>
-                </c14:spPr>
-              </c14:invertSolidFillFmt>
-            </c:ext>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-9326-4A8A-AD6D-972A1E0DBE4A}"/>
+              <c16:uniqueId val="{00000000-5417-431E-B3D1-D106FC7FDDBC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -966,7 +1272,7 @@
         <xdr:cNvPr id="2" name="Chart">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1007,7 +1313,7 @@
         <xdr:cNvPr id="2" name="Chart">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1223,6 +1529,807 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="2" width="25" customWidth="1"/>
+    <col min="3" max="3" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A1" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+    </row>
+    <row r="2" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+    </row>
+    <row r="3" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A3" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+    </row>
+    <row r="4" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A4" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+    </row>
+    <row r="5" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A5" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="20"/>
+      <c r="C5" s="20"/>
+    </row>
+    <row r="6" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A6" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+    </row>
+    <row r="7" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A16" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A19" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+    </row>
+    <row r="24" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+    </row>
+    <row r="25" spans="1:3" ht="30.1" customHeight="1">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1">
+      <c r="A2" s="17">
+        <v>2</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1">
+      <c r="A3" s="17">
+        <v>3</v>
+      </c>
+      <c r="C3" s="21"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1">
+      <c r="A4" s="17">
+        <v>2</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="25" customHeight="1">
+      <c r="A5" s="17">
+        <v>1</v>
+      </c>
+      <c r="C5" s="21"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1">
+      <c r="A6" s="17">
+        <v>4</v>
+      </c>
+      <c r="C6" s="21"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1">
+      <c r="A7" s="17">
+        <v>3</v>
+      </c>
+      <c r="C7" s="21"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1">
+      <c r="A8" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1">
+      <c r="A9" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="25" customHeight="1">
+      <c r="A10" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="25" customHeight="1">
+      <c r="A11" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="25" customHeight="1">
+      <c r="A12" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="25" customHeight="1">
+      <c r="A13" s="17">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" customHeight="1">
+      <c r="A2" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="17">
+        <v>9</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1">
+      <c r="A3" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B3" s="17">
+        <v>11</v>
+      </c>
+      <c r="D3" s="21"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1">
+      <c r="A4" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="B4" s="17">
+        <v>5</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="D5" s="21"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="D6" s="21"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="D7" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="3" width="22" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1">
+      <c r="A2" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="B2" s="17">
+        <v>12</v>
+      </c>
+      <c r="C2" s="17">
+        <v>20</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1">
+      <c r="A3" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="17">
+        <v>14</v>
+      </c>
+      <c r="C3" s="17">
+        <v>20</v>
+      </c>
+      <c r="E3" s="21"/>
+    </row>
+    <row r="4" spans="1:5" ht="25" customHeight="1">
+      <c r="A4" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" s="17">
+        <v>6</v>
+      </c>
+      <c r="C4" s="17">
+        <v>20</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="E5" s="21"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="E6" s="21"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="E7" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1">
+      <c r="A2" s="17">
+        <v>0</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1">
+      <c r="A3" s="17">
+        <v>1</v>
+      </c>
+      <c r="C3" s="21"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1">
+      <c r="A4" s="17">
+        <v>1</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="25" customHeight="1">
+      <c r="A5" s="17">
+        <v>2</v>
+      </c>
+      <c r="C5" s="21"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1">
+      <c r="A6" s="17">
+        <v>2</v>
+      </c>
+      <c r="C6" s="21"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1">
+      <c r="A7" s="17">
+        <v>2</v>
+      </c>
+      <c r="C7" s="21"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1">
+      <c r="A8" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1">
+      <c r="A9" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="25" customHeight="1">
+      <c r="A10" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="25" customHeight="1">
+      <c r="A11" s="17">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1">
+      <c r="A2" s="17">
+        <v>5</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1">
+      <c r="A3" s="17">
+        <v>5.5</v>
+      </c>
+      <c r="C3" s="21"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1">
+      <c r="A4" s="17">
+        <v>6</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="25" customHeight="1">
+      <c r="A5" s="17">
+        <v>6</v>
+      </c>
+      <c r="C5" s="21"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1">
+      <c r="A6" s="17">
+        <v>6.5</v>
+      </c>
+      <c r="C6" s="21"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1">
+      <c r="A7" s="17">
+        <v>7</v>
+      </c>
+      <c r="C7" s="21"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1">
+      <c r="A8" s="17">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1">
+      <c r="A9" s="17">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" customHeight="1">
+      <c r="A2" s="17">
+        <v>2</v>
+      </c>
+      <c r="B2" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1">
+      <c r="A3" s="17">
+        <v>3</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="D3" s="21"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1">
+      <c r="A4" s="17">
+        <v>4</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="D5" s="21"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="D6" s="21"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="D7" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="3" width="22" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1">
+      <c r="A2" s="17" t="s">
+        <v>177</v>
+      </c>
+      <c r="B2" s="17">
+        <v>30</v>
+      </c>
+      <c r="C2" s="17">
+        <v>40</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1">
+      <c r="A3" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="B3" s="17">
+        <v>32</v>
+      </c>
+      <c r="C3" s="17">
+        <v>80</v>
+      </c>
+      <c r="E3" s="21"/>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="E4" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="E5" s="21"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="E6" s="21"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="E7" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Q40"/>
   <sheetFormatPr defaultRowHeight="13.6"/>
   <cols>
@@ -1233,7 +2340,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="22.1" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1255,7 +2362,7 @@
     <row r="2" spans="1:17" ht="22.1" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="C2" s="1">
         <f>COUNT(Data!E2:E37)</f>
@@ -1296,29 +2403,29 @@
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17" ht="36" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>9</v>
+      <c r="A4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
@@ -1335,29 +2442,29 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="6">
+        <v>60</v>
+      </c>
+      <c r="C5" s="8">
         <f>COUNTIFS(Data!$E$2:$E$37,A5)</f>
         <v>4</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="9">
         <f>C5/$C$2</f>
         <v>0.1111111111111111</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="10">
         <f>D5</f>
         <v>0.1111111111111111</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="8">
         <f>SUM($C$5:C5)</f>
         <v>4</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="9">
         <f>F5/$C$2</f>
         <v>0.1111111111111111</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="10">
         <f>G5</f>
         <v>0.1111111111111111</v>
       </c>
@@ -1376,29 +2483,29 @@
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="6">
+        <v>61</v>
+      </c>
+      <c r="C6" s="8">
         <f>COUNTIFS(Data!$E$2:$E$37,A6)</f>
         <v>10</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="9">
         <f>C6/$C$2</f>
         <v>0.27777777777777779</v>
       </c>
-      <c r="E6" s="8">
+      <c r="E6" s="10">
         <f>D6</f>
         <v>0.27777777777777779</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="8">
         <f>SUM($C$5:C6)</f>
         <v>14</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="9">
         <f>F6/$C$2</f>
         <v>0.3888888888888889</v>
       </c>
-      <c r="H6" s="8">
+      <c r="H6" s="10">
         <f>G6</f>
         <v>0.3888888888888889</v>
       </c>
@@ -1417,29 +2524,29 @@
         <v>3</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="6">
+        <v>62</v>
+      </c>
+      <c r="C7" s="8">
         <f>COUNTIFS(Data!$E$2:$E$37,A7)</f>
         <v>14</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="9">
         <f>C7/$C$2</f>
         <v>0.3888888888888889</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="10">
         <f>D7</f>
         <v>0.3888888888888889</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="8">
         <f>SUM($C$5:C7)</f>
         <v>28</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="9">
         <f>F7/$C$2</f>
         <v>0.77777777777777779</v>
       </c>
-      <c r="H7" s="8">
+      <c r="H7" s="10">
         <f>G7</f>
         <v>0.77777777777777779</v>
       </c>
@@ -1458,29 +2565,29 @@
         <v>4</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="6">
+        <v>63</v>
+      </c>
+      <c r="C8" s="8">
         <f>COUNTIFS(Data!$E$2:$E$37,A8)</f>
         <v>8</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="9">
         <f>C8/$C$2</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="10">
         <f>D8</f>
         <v>0.22222222222222221</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="8">
         <f>SUM($C$5:C8)</f>
         <v>36</v>
       </c>
-      <c r="G8" s="7">
+      <c r="G8" s="9">
         <f>F8/$C$2</f>
         <v>1</v>
       </c>
-      <c r="H8" s="8">
+      <c r="H8" s="10">
         <f>G8</f>
         <v>1</v>
       </c>
@@ -1498,8 +2605,8 @@
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="5"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="7"/>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
@@ -1515,18 +2622,18 @@
     </row>
     <row r="10" spans="1:17" ht="22.1" customHeight="1">
       <c r="A10" s="1"/>
-      <c r="B10" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="9">
+      <c r="B10" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="11">
         <f>SUM(C5:C8)</f>
         <v>36</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="12">
         <f>SUM(D5:D8)</f>
         <v>1</v>
       </c>
-      <c r="E10" s="11">
+      <c r="E10" s="13">
         <f>D10</f>
         <v>1</v>
       </c>
@@ -1563,8 +2670,8 @@
       <c r="Q11" s="1"/>
     </row>
     <row r="12" spans="1:17" ht="22.1" customHeight="1">
-      <c r="A12" s="12" t="s">
-        <v>15</v>
+      <c r="A12" s="14" t="s">
+        <v>65</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -1584,8 +2691,8 @@
       <c r="Q12" s="1"/>
     </row>
     <row r="13" spans="1:17" ht="22.1" customHeight="1">
-      <c r="A13" s="12" t="s">
-        <v>16</v>
+      <c r="A13" s="14" t="s">
+        <v>66</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -1624,8 +2731,8 @@
       <c r="Q14" s="1"/>
     </row>
     <row r="15" spans="1:17" ht="22.1" customHeight="1">
-      <c r="A15" s="12" t="s">
-        <v>17</v>
+      <c r="A15" s="14" t="s">
+        <v>67</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2125,8 +3232,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q40"/>
   <sheetFormatPr defaultRowHeight="13.6"/>
   <cols>
@@ -2138,7 +3245,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="22.1" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2160,7 +3267,7 @@
     <row r="2" spans="1:17" ht="22.1" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="C2" s="1">
         <f>COUNT(Data!B2:B37)</f>
@@ -2201,23 +3308,23 @@
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:17" ht="36" customHeight="1">
-      <c r="A4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>6</v>
+      <c r="A4" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>56</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -2239,17 +3346,17 @@
         <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D5" s="6">
+        <v>73</v>
+      </c>
+      <c r="D5" s="8">
         <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A5,Data!$B$2:$B$37,"&lt;="&amp;B5)</f>
         <v>3</v>
       </c>
-      <c r="E5" s="7">
+      <c r="E5" s="9">
         <f t="shared" ref="E5:E10" si="0">D5/$C$2</f>
         <v>9.0909090909090912E-2</v>
       </c>
-      <c r="F5" s="8">
+      <c r="F5" s="10">
         <f t="shared" ref="F5:F10" si="1">E5</f>
         <v>9.0909090909090912E-2</v>
       </c>
@@ -2273,17 +3380,17 @@
         <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D6" s="6">
+        <v>74</v>
+      </c>
+      <c r="D6" s="8">
         <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A6,Data!$B$2:$B$37,"&lt;="&amp;B6)</f>
         <v>5</v>
       </c>
-      <c r="E6" s="7">
+      <c r="E6" s="9">
         <f t="shared" si="0"/>
         <v>0.15151515151515152</v>
       </c>
-      <c r="F6" s="8">
+      <c r="F6" s="10">
         <f t="shared" si="1"/>
         <v>0.15151515151515152</v>
       </c>
@@ -2307,17 +3414,17 @@
         <v>7</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D7" s="6">
+        <v>75</v>
+      </c>
+      <c r="D7" s="8">
         <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A7,Data!$B$2:$B$37,"&lt;="&amp;B7)</f>
         <v>8</v>
       </c>
-      <c r="E7" s="7">
+      <c r="E7" s="9">
         <f t="shared" si="0"/>
         <v>0.24242424242424243</v>
       </c>
-      <c r="F7" s="8">
+      <c r="F7" s="10">
         <f t="shared" si="1"/>
         <v>0.24242424242424243</v>
       </c>
@@ -2341,17 +3448,17 @@
         <v>8</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D8" s="6">
+        <v>76</v>
+      </c>
+      <c r="D8" s="8">
         <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A8,Data!$B$2:$B$37,"&lt;="&amp;B8)</f>
         <v>10</v>
       </c>
-      <c r="E8" s="7">
+      <c r="E8" s="9">
         <f t="shared" si="0"/>
         <v>0.30303030303030304</v>
       </c>
-      <c r="F8" s="8">
+      <c r="F8" s="10">
         <f t="shared" si="1"/>
         <v>0.30303030303030304</v>
       </c>
@@ -2375,17 +3482,17 @@
         <v>9</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D9" s="6">
+        <v>77</v>
+      </c>
+      <c r="D9" s="8">
         <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A9,Data!$B$2:$B$37,"&lt;="&amp;B9)</f>
         <v>5</v>
       </c>
-      <c r="E9" s="7">
+      <c r="E9" s="9">
         <f t="shared" si="0"/>
         <v>0.15151515151515152</v>
       </c>
-      <c r="F9" s="8">
+      <c r="F9" s="10">
         <f t="shared" si="1"/>
         <v>0.15151515151515152</v>
       </c>
@@ -2409,17 +3516,17 @@
         <v>10</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D10" s="6">
+        <v>78</v>
+      </c>
+      <c r="D10" s="8">
         <f>COUNTIFS(Data!$B$2:$B$37,"&gt;"&amp;A10,Data!$B$2:$B$37,"&lt;="&amp;B10)</f>
         <v>2</v>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="9">
         <f t="shared" si="0"/>
         <v>6.0606060606060608E-2</v>
       </c>
-      <c r="F10" s="8">
+      <c r="F10" s="10">
         <f t="shared" si="1"/>
         <v>6.0606060606060608E-2</v>
       </c>
@@ -2440,8 +3547,8 @@
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="5"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="7"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -2457,18 +3564,18 @@
     <row r="12" spans="1:17" ht="22.1" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="9">
+      <c r="C12" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="11">
         <f>SUM(D5:D10)</f>
         <v>33</v>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="12">
         <f>SUM(E5:E10)</f>
         <v>1</v>
       </c>
-      <c r="F12" s="11">
+      <c r="F12" s="13">
         <f>E12</f>
         <v>1</v>
       </c>
@@ -2504,8 +3611,8 @@
       <c r="Q13" s="1"/>
     </row>
     <row r="14" spans="1:17" ht="22.1" customHeight="1">
-      <c r="A14" s="12" t="s">
-        <v>86</v>
+      <c r="A14" s="14" t="s">
+        <v>79</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -2525,8 +3632,8 @@
       <c r="Q14" s="1"/>
     </row>
     <row r="15" spans="1:17" ht="22.1" customHeight="1">
-      <c r="A15" s="12" t="s">
-        <v>23</v>
+      <c r="A15" s="14" t="s">
+        <v>80</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
@@ -2565,8 +3672,8 @@
       <c r="Q16" s="1"/>
     </row>
     <row r="17" spans="1:17" ht="22.1" customHeight="1">
-      <c r="A17" s="12" t="s">
-        <v>24</v>
+      <c r="A17" s="14" t="s">
+        <v>81</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -2586,8 +3693,8 @@
       <c r="Q17" s="1"/>
     </row>
     <row r="18" spans="1:17" ht="22.1" customHeight="1">
-      <c r="A18" s="12" t="s">
-        <v>25</v>
+      <c r="A18" s="14" t="s">
+        <v>82</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -3030,8 +4137,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:Q40"/>
   <sheetFormatPr defaultRowHeight="13.6"/>
   <cols>
@@ -3041,24 +4148,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="36" customHeight="1">
-      <c r="A1" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>30</v>
+      <c r="A1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1" t="s">
-        <v>31</v>
+        <v>88</v>
       </c>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
@@ -3073,18 +4180,18 @@
     </row>
     <row r="2" spans="1:17" ht="22.1" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="13">
+        <v>89</v>
+      </c>
+      <c r="B2" s="15">
         <v>6</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="16">
         <v>5</v>
       </c>
-      <c r="D2" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" s="14">
+      <c r="D2" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="16">
         <v>2</v>
       </c>
       <c r="F2" s="1"/>
@@ -3102,23 +4209,23 @@
     </row>
     <row r="3" spans="1:17" ht="22.1" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B3" s="13">
+        <v>91</v>
+      </c>
+      <c r="B3" s="15">
         <v>8</v>
       </c>
-      <c r="C3" s="14">
+      <c r="C3" s="16">
         <v>9</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E3" s="14">
+      <c r="D3" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="16">
         <v>4</v>
       </c>
       <c r="F3" s="1"/>
-      <c r="G3" s="12" t="s">
-        <v>36</v>
+      <c r="G3" s="14" t="s">
+        <v>93</v>
       </c>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -3133,23 +4240,23 @@
     </row>
     <row r="4" spans="1:17" ht="22.1" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="13">
+        <v>94</v>
+      </c>
+      <c r="B4" s="15">
         <v>7</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="16">
         <v>8</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E4" s="14">
+      <c r="D4" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="16">
         <v>3</v>
       </c>
       <c r="F4" s="1"/>
-      <c r="G4" s="12" t="s">
-        <v>38</v>
+      <c r="G4" s="14" t="s">
+        <v>95</v>
       </c>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
@@ -3164,23 +4271,23 @@
     </row>
     <row r="5" spans="1:17" ht="22.1" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="13">
+        <v>96</v>
+      </c>
+      <c r="B5" s="15">
         <v>5</v>
       </c>
-      <c r="C5" s="14">
+      <c r="C5" s="16">
         <v>6</v>
       </c>
-      <c r="D5" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E5" s="14">
+      <c r="D5" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" s="16">
         <v>2</v>
       </c>
       <c r="F5" s="1"/>
-      <c r="G5" s="12" t="s">
-        <v>40</v>
+      <c r="G5" s="14" t="s">
+        <v>97</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -3195,21 +4302,21 @@
     </row>
     <row r="6" spans="1:17" ht="22.1" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="14">
+        <v>98</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="16">
         <v>7</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="14">
+      <c r="D6" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="16">
         <v>3</v>
       </c>
       <c r="F6" s="1"/>
-      <c r="G6" s="12" t="s">
-        <v>42</v>
+      <c r="G6" s="14" t="s">
+        <v>99</v>
       </c>
       <c r="H6" s="1"/>
       <c r="I6" s="1"/>
@@ -3224,23 +4331,23 @@
     </row>
     <row r="7" spans="1:17" ht="22.1" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="13">
+        <v>100</v>
+      </c>
+      <c r="B7" s="15">
         <v>7</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="16">
         <v>0</v>
       </c>
-      <c r="D7" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="14">
+      <c r="D7" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E7" s="16">
         <v>1</v>
       </c>
       <c r="F7" s="1"/>
-      <c r="G7" s="12" t="s">
-        <v>44</v>
+      <c r="G7" s="14" t="s">
+        <v>101</v>
       </c>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
@@ -3255,23 +4362,23 @@
     </row>
     <row r="8" spans="1:17" ht="22.1" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="13">
+        <v>102</v>
+      </c>
+      <c r="B8" s="15">
         <v>4.5</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="16">
         <v>2</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="14">
+      <c r="D8" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E8" s="16">
         <v>1</v>
       </c>
       <c r="F8" s="1"/>
-      <c r="G8" s="12" t="s">
-        <v>46</v>
+      <c r="G8" s="14" t="s">
+        <v>103</v>
       </c>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
@@ -3286,23 +4393,23 @@
     </row>
     <row r="9" spans="1:17" ht="22.1" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B9" s="13">
+        <v>104</v>
+      </c>
+      <c r="B9" s="15">
         <v>6.3</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="16">
         <v>7</v>
       </c>
-      <c r="D9" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="14">
+      <c r="D9" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E9" s="16">
         <v>3</v>
       </c>
       <c r="F9" s="1"/>
-      <c r="G9" s="12" t="s">
-        <v>48</v>
+      <c r="G9" s="14" t="s">
+        <v>105</v>
       </c>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
@@ -3317,23 +4424,23 @@
     </row>
     <row r="10" spans="1:17" ht="22.1" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="13">
+        <v>106</v>
+      </c>
+      <c r="B10" s="15">
         <v>7.3</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="16">
         <v>9</v>
       </c>
-      <c r="D10" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E10" s="14">
+      <c r="D10" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E10" s="16">
         <v>4</v>
       </c>
       <c r="F10" s="1"/>
-      <c r="G10" s="12" t="s">
-        <v>50</v>
+      <c r="G10" s="14" t="s">
+        <v>107</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -3348,23 +4455,23 @@
     </row>
     <row r="11" spans="1:17" ht="22.1" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" s="13">
+        <v>108</v>
+      </c>
+      <c r="B11" s="15">
         <v>8.1</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="16">
         <v>4</v>
       </c>
-      <c r="D11" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="14">
+      <c r="D11" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E11" s="16">
         <v>2</v>
       </c>
       <c r="F11" s="1"/>
-      <c r="G11" s="12" t="s">
-        <v>52</v>
+      <c r="G11" s="14" t="s">
+        <v>109</v>
       </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
@@ -3379,21 +4486,21 @@
     </row>
     <row r="12" spans="1:17" ht="22.1" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="14">
+        <v>110</v>
+      </c>
+      <c r="B12" s="15"/>
+      <c r="C12" s="16">
         <v>7</v>
       </c>
-      <c r="D12" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" s="14">
+      <c r="D12" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E12" s="16">
         <v>3</v>
       </c>
       <c r="F12" s="1"/>
-      <c r="G12" s="12" t="s">
-        <v>54</v>
+      <c r="G12" s="14" t="s">
+        <v>111</v>
       </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
@@ -3408,18 +4515,18 @@
     </row>
     <row r="13" spans="1:17" ht="22.1" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B13" s="13">
+        <v>112</v>
+      </c>
+      <c r="B13" s="15">
         <v>6</v>
       </c>
-      <c r="C13" s="14">
+      <c r="C13" s="16">
         <v>10</v>
       </c>
-      <c r="D13" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E13" s="14">
+      <c r="D13" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E13" s="16">
         <v>2</v>
       </c>
       <c r="F13" s="1"/>
@@ -3437,18 +4544,18 @@
     </row>
     <row r="14" spans="1:17" ht="22.1" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B14" s="13">
+        <v>113</v>
+      </c>
+      <c r="B14" s="15">
         <v>7.1</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="16">
         <v>5</v>
       </c>
-      <c r="D14" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E14" s="14">
+      <c r="D14" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="16">
         <v>3</v>
       </c>
       <c r="F14" s="1"/>
@@ -3466,18 +4573,18 @@
     </row>
     <row r="15" spans="1:17" ht="22.1" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B15" s="13">
+        <v>114</v>
+      </c>
+      <c r="B15" s="15">
         <v>7.9</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="16">
         <v>8</v>
       </c>
-      <c r="D15" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E15" s="14">
+      <c r="D15" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" s="16">
         <v>1</v>
       </c>
       <c r="F15" s="1"/>
@@ -3495,18 +4602,18 @@
     </row>
     <row r="16" spans="1:17" ht="22.1" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B16" s="13">
+        <v>115</v>
+      </c>
+      <c r="B16" s="15">
         <v>9.1999999999999993</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="16">
         <v>11</v>
       </c>
-      <c r="D16" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E16" s="14">
+      <c r="D16" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E16" s="16">
         <v>3</v>
       </c>
       <c r="F16" s="1"/>
@@ -3524,18 +4631,18 @@
     </row>
     <row r="17" spans="1:17" ht="22.1" customHeight="1">
       <c r="A17" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B17" s="13">
+        <v>116</v>
+      </c>
+      <c r="B17" s="15">
         <v>5.5</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="16">
         <v>6</v>
       </c>
-      <c r="D17" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="14">
+      <c r="D17" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E17" s="16">
         <v>4</v>
       </c>
       <c r="F17" s="1"/>
@@ -3553,18 +4660,18 @@
     </row>
     <row r="18" spans="1:17" ht="22.1" customHeight="1">
       <c r="A18" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="13">
+        <v>117</v>
+      </c>
+      <c r="B18" s="15">
         <v>6.8</v>
       </c>
-      <c r="C18" s="14">
+      <c r="C18" s="16">
         <v>8</v>
       </c>
-      <c r="D18" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E18" s="14">
+      <c r="D18" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="16">
         <v>2</v>
       </c>
       <c r="F18" s="1"/>
@@ -3582,18 +4689,18 @@
     </row>
     <row r="19" spans="1:17" ht="22.1" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="B19" s="13">
+        <v>118</v>
+      </c>
+      <c r="B19" s="15">
         <v>7.5</v>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="16">
         <v>3</v>
       </c>
-      <c r="D19" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E19" s="14">
+      <c r="D19" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E19" s="16">
         <v>4</v>
       </c>
       <c r="F19" s="1"/>
@@ -3611,18 +4718,18 @@
     </row>
     <row r="20" spans="1:17" ht="22.1" customHeight="1">
       <c r="A20" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="13">
+        <v>119</v>
+      </c>
+      <c r="B20" s="15">
         <v>8.8000000000000007</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="16">
         <v>7</v>
       </c>
-      <c r="D20" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E20" s="14">
+      <c r="D20" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" s="16">
         <v>2</v>
       </c>
       <c r="F20" s="1"/>
@@ -3640,18 +4747,18 @@
     </row>
     <row r="21" spans="1:17" ht="22.1" customHeight="1">
       <c r="A21" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="B21" s="13">
+        <v>120</v>
+      </c>
+      <c r="B21" s="15">
         <v>4.8</v>
       </c>
-      <c r="C21" s="14">
+      <c r="C21" s="16">
         <v>9</v>
       </c>
-      <c r="D21" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E21" s="14">
+      <c r="D21" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="16">
         <v>3</v>
       </c>
       <c r="F21" s="1"/>
@@ -3669,18 +4776,18 @@
     </row>
     <row r="22" spans="1:17" ht="22.1" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="B22" s="13">
+        <v>121</v>
+      </c>
+      <c r="B22" s="15">
         <v>6.5</v>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="16">
         <v>5</v>
       </c>
-      <c r="D22" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E22" s="14">
+      <c r="D22" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E22" s="16">
         <v>1</v>
       </c>
       <c r="F22" s="1"/>
@@ -3698,18 +4805,18 @@
     </row>
     <row r="23" spans="1:17" ht="22.1" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="B23" s="13">
+        <v>122</v>
+      </c>
+      <c r="B23" s="15">
         <v>7.4</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="16">
         <v>7</v>
       </c>
-      <c r="D23" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E23" s="14">
+      <c r="D23" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E23" s="16">
         <v>3</v>
       </c>
       <c r="F23" s="1"/>
@@ -3727,18 +4834,18 @@
     </row>
     <row r="24" spans="1:17" ht="22.1" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B24" s="13">
+        <v>123</v>
+      </c>
+      <c r="B24" s="15">
         <v>8.3000000000000007</v>
       </c>
-      <c r="C24" s="14">
+      <c r="C24" s="16">
         <v>10</v>
       </c>
-      <c r="D24" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E24" s="14">
+      <c r="D24" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E24" s="16">
         <v>4</v>
       </c>
       <c r="F24" s="1"/>
@@ -3756,16 +4863,16 @@
     </row>
     <row r="25" spans="1:17" ht="22.1" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="14">
+        <v>124</v>
+      </c>
+      <c r="B25" s="15"/>
+      <c r="C25" s="16">
         <v>6</v>
       </c>
-      <c r="D25" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E25" s="14">
+      <c r="D25" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E25" s="16">
         <v>3</v>
       </c>
       <c r="F25" s="1"/>
@@ -3783,18 +4890,18 @@
     </row>
     <row r="26" spans="1:17" ht="22.1" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" s="13">
+        <v>125</v>
+      </c>
+      <c r="B26" s="15">
         <v>6.2</v>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="16">
         <v>8</v>
       </c>
-      <c r="D26" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E26" s="14">
+      <c r="D26" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E26" s="16">
         <v>4</v>
       </c>
       <c r="F26" s="1"/>
@@ -3812,18 +4919,18 @@
     </row>
     <row r="27" spans="1:17" ht="22.1" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B27" s="13">
+        <v>126</v>
+      </c>
+      <c r="B27" s="15">
         <v>7.2</v>
       </c>
-      <c r="C27" s="14">
+      <c r="C27" s="16">
         <v>12</v>
       </c>
-      <c r="D27" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E27" s="14">
+      <c r="D27" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E27" s="16">
         <v>2</v>
       </c>
       <c r="F27" s="1"/>
@@ -3841,18 +4948,18 @@
     </row>
     <row r="28" spans="1:17" ht="22.1" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B28" s="13">
+        <v>127</v>
+      </c>
+      <c r="B28" s="15">
         <v>8</v>
       </c>
-      <c r="C28" s="14">
+      <c r="C28" s="16">
         <v>6</v>
       </c>
-      <c r="D28" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E28" s="14">
+      <c r="D28" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E28" s="16">
         <v>3</v>
       </c>
       <c r="F28" s="1"/>
@@ -3870,18 +4977,18 @@
     </row>
     <row r="29" spans="1:17" ht="22.1" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B29" s="13">
+        <v>128</v>
+      </c>
+      <c r="B29" s="15">
         <v>9.5</v>
       </c>
-      <c r="C29" s="14">
+      <c r="C29" s="16">
         <v>9</v>
       </c>
-      <c r="D29" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E29" s="14">
+      <c r="D29" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E29" s="16">
         <v>2</v>
       </c>
       <c r="F29" s="1"/>
@@ -3899,18 +5006,18 @@
     </row>
     <row r="30" spans="1:17" ht="22.1" customHeight="1">
       <c r="A30" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30" s="13">
+        <v>129</v>
+      </c>
+      <c r="B30" s="15">
         <v>5.8</v>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="16">
         <v>4</v>
       </c>
-      <c r="D30" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E30" s="14">
+      <c r="D30" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" s="16">
         <v>3</v>
       </c>
       <c r="F30" s="1"/>
@@ -3928,18 +5035,18 @@
     </row>
     <row r="31" spans="1:17" ht="22.1" customHeight="1">
       <c r="A31" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B31" s="13">
+        <v>130</v>
+      </c>
+      <c r="B31" s="15">
         <v>7</v>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="16">
         <v>7</v>
       </c>
-      <c r="D31" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E31" s="14">
+      <c r="D31" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E31" s="16">
         <v>4</v>
       </c>
       <c r="F31" s="1"/>
@@ -3957,18 +5064,18 @@
     </row>
     <row r="32" spans="1:17" ht="22.1" customHeight="1">
       <c r="A32" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B32" s="13">
+        <v>131</v>
+      </c>
+      <c r="B32" s="15">
         <v>7.7</v>
       </c>
-      <c r="C32" s="14">
+      <c r="C32" s="16">
         <v>10</v>
       </c>
-      <c r="D32" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E32" s="14">
+      <c r="D32" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E32" s="16">
         <v>3</v>
       </c>
       <c r="F32" s="1"/>
@@ -3986,18 +5093,18 @@
     </row>
     <row r="33" spans="1:17" ht="22.1" customHeight="1">
       <c r="A33" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="B33" s="13">
+        <v>132</v>
+      </c>
+      <c r="B33" s="15">
         <v>9</v>
       </c>
-      <c r="C33" s="14">
+      <c r="C33" s="16">
         <v>5</v>
       </c>
-      <c r="D33" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E33" s="14">
+      <c r="D33" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E33" s="16">
         <v>4</v>
       </c>
       <c r="F33" s="1"/>
@@ -4015,18 +5122,18 @@
     </row>
     <row r="34" spans="1:17" ht="22.1" customHeight="1">
       <c r="A34" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B34" s="13">
+        <v>133</v>
+      </c>
+      <c r="B34" s="15">
         <v>5.2</v>
       </c>
-      <c r="C34" s="14">
+      <c r="C34" s="16">
         <v>8</v>
       </c>
-      <c r="D34" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E34" s="14">
+      <c r="D34" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E34" s="16">
         <v>2</v>
       </c>
       <c r="F34" s="1"/>
@@ -4044,18 +5151,18 @@
     </row>
     <row r="35" spans="1:17" ht="22.1" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B35" s="13">
+        <v>134</v>
+      </c>
+      <c r="B35" s="15">
         <v>6.5</v>
       </c>
-      <c r="C35" s="14">
+      <c r="C35" s="16">
         <v>11</v>
       </c>
-      <c r="D35" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="E35" s="14">
+      <c r="D35" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="E35" s="16">
         <v>3</v>
       </c>
       <c r="F35" s="1"/>
@@ -4073,18 +5180,18 @@
     </row>
     <row r="36" spans="1:17" ht="22.1" customHeight="1">
       <c r="A36" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B36" s="13">
+        <v>135</v>
+      </c>
+      <c r="B36" s="15">
         <v>7.5</v>
       </c>
-      <c r="C36" s="14">
+      <c r="C36" s="16">
         <v>6</v>
       </c>
-      <c r="D36" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E36" s="14">
+      <c r="D36" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E36" s="16">
         <v>2</v>
       </c>
       <c r="F36" s="1"/>
@@ -4102,18 +5209,18 @@
     </row>
     <row r="37" spans="1:17" ht="22.1" customHeight="1">
       <c r="A37" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B37" s="13">
+        <v>136</v>
+      </c>
+      <c r="B37" s="15">
         <v>8.5</v>
       </c>
-      <c r="C37" s="14">
+      <c r="C37" s="16">
         <v>8</v>
       </c>
-      <c r="D37" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="E37" s="14">
+      <c r="D37" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="E37" s="16">
         <v>3</v>
       </c>
       <c r="F37" s="1"/>
@@ -4188,15 +5295,754 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="whole" sqref="E2:E37" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="whole" sqref="E2:E37" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>1</formula1>
       <formula2>4</formula2>
     </dataValidation>
-    <dataValidation type="whole" sqref="C2:C37" xr:uid="{00000000-0002-0000-0200-000001000000}">
+    <dataValidation type="whole" sqref="C2:C37" xr:uid="{00000000-0002-0000-0300-000001000000}">
       <formula1>0</formula1>
       <formula2>12</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="5" width="22" customWidth="1"/>
+    <col min="7" max="7" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="25" customHeight="1">
+      <c r="A2" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="17">
+        <v>6</v>
+      </c>
+      <c r="C2" s="17">
+        <v>5</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E2" s="17">
+        <v>2</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="25" customHeight="1">
+      <c r="A3" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B3" s="17">
+        <v>8</v>
+      </c>
+      <c r="C3" s="17">
+        <v>9</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3" s="17">
+        <v>4</v>
+      </c>
+      <c r="G3" s="21"/>
+    </row>
+    <row r="4" spans="1:7" ht="25" customHeight="1">
+      <c r="A4" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" s="17">
+        <v>7</v>
+      </c>
+      <c r="C4" s="17">
+        <v>8</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" s="17">
+        <v>3</v>
+      </c>
+      <c r="G4" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="25" customHeight="1">
+      <c r="A5" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" s="17">
+        <v>5</v>
+      </c>
+      <c r="C5" s="17">
+        <v>6</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" s="17">
+        <v>2</v>
+      </c>
+      <c r="G5" s="21"/>
+    </row>
+    <row r="6" spans="1:7" ht="25" customHeight="1">
+      <c r="A6" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17">
+        <v>7</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="17">
+        <v>3</v>
+      </c>
+      <c r="G6" s="21"/>
+    </row>
+    <row r="7" spans="1:7" ht="25" customHeight="1">
+      <c r="A7" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" s="17">
+        <v>7</v>
+      </c>
+      <c r="C7" s="17">
+        <v>0</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>92</v>
+      </c>
+      <c r="E7" s="17">
+        <v>1</v>
+      </c>
+      <c r="G7" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="G4:G7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="2" width="22" customWidth="1"/>
+    <col min="4" max="4" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" customHeight="1">
+      <c r="A2" s="17" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="17">
+        <v>14</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="25" customHeight="1">
+      <c r="A3" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" s="17">
+        <v>12</v>
+      </c>
+      <c r="D3" s="21"/>
+    </row>
+    <row r="4" spans="1:4" ht="25" customHeight="1">
+      <c r="A4" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4" s="17">
+        <v>10</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="D5" s="21"/>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="D6" s="21"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="D7" s="21"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="D4:D7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="7" width="22" customWidth="1"/>
+    <col min="9" max="9" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="I1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="25" customHeight="1">
+      <c r="A2" s="17">
+        <v>1</v>
+      </c>
+      <c r="B2" s="17">
+        <v>1</v>
+      </c>
+      <c r="C2" s="17">
+        <v>1</v>
+      </c>
+      <c r="D2" s="17">
+        <v>1</v>
+      </c>
+      <c r="E2" s="17">
+        <v>1</v>
+      </c>
+      <c r="F2" s="17">
+        <v>4</v>
+      </c>
+      <c r="G2" s="17">
+        <v>1</v>
+      </c>
+      <c r="I2" s="21" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="25" customHeight="1">
+      <c r="A3" s="17">
+        <v>2</v>
+      </c>
+      <c r="B3" s="17">
+        <v>2</v>
+      </c>
+      <c r="C3" s="17">
+        <v>3</v>
+      </c>
+      <c r="D3" s="17">
+        <v>1</v>
+      </c>
+      <c r="E3" s="17">
+        <v>6</v>
+      </c>
+      <c r="F3" s="17">
+        <v>4</v>
+      </c>
+      <c r="G3" s="17">
+        <v>3</v>
+      </c>
+      <c r="I3" s="21"/>
+    </row>
+    <row r="4" spans="1:9" ht="25" customHeight="1">
+      <c r="A4" s="17">
+        <v>3</v>
+      </c>
+      <c r="B4" s="17">
+        <v>4</v>
+      </c>
+      <c r="C4" s="17">
+        <v>10</v>
+      </c>
+      <c r="D4" s="17">
+        <v>2</v>
+      </c>
+      <c r="E4" s="17">
+        <v>10</v>
+      </c>
+      <c r="F4" s="17">
+        <v>4</v>
+      </c>
+      <c r="G4" s="17">
+        <v>8</v>
+      </c>
+      <c r="I4" s="21" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="25" customHeight="1">
+      <c r="A5" s="17">
+        <v>4</v>
+      </c>
+      <c r="B5" s="17">
+        <v>7</v>
+      </c>
+      <c r="C5" s="17">
+        <v>8</v>
+      </c>
+      <c r="D5" s="17">
+        <v>3</v>
+      </c>
+      <c r="E5" s="17">
+        <v>4</v>
+      </c>
+      <c r="F5" s="17">
+        <v>4</v>
+      </c>
+      <c r="G5" s="17">
+        <v>9</v>
+      </c>
+      <c r="I5" s="21"/>
+    </row>
+    <row r="6" spans="1:9" ht="25" customHeight="1">
+      <c r="A6" s="17">
+        <v>5</v>
+      </c>
+      <c r="B6" s="17">
+        <v>10</v>
+      </c>
+      <c r="C6" s="17">
+        <v>5</v>
+      </c>
+      <c r="D6" s="17">
+        <v>5</v>
+      </c>
+      <c r="E6" s="17">
+        <v>1</v>
+      </c>
+      <c r="F6" s="17">
+        <v>4</v>
+      </c>
+      <c r="G6" s="17">
+        <v>4</v>
+      </c>
+      <c r="I6" s="21"/>
+    </row>
+    <row r="7" spans="1:9" ht="25" customHeight="1">
+      <c r="A7" s="17">
+        <v>6</v>
+      </c>
+      <c r="B7" s="17">
+        <v>7</v>
+      </c>
+      <c r="C7" s="17">
+        <v>3</v>
+      </c>
+      <c r="D7" s="17">
+        <v>8</v>
+      </c>
+      <c r="E7" s="17">
+        <v>4</v>
+      </c>
+      <c r="F7" s="17">
+        <v>4</v>
+      </c>
+      <c r="G7" s="17">
+        <v>1</v>
+      </c>
+      <c r="I7" s="21"/>
+    </row>
+    <row r="8" spans="1:9" ht="25" customHeight="1">
+      <c r="A8" s="17">
+        <v>7</v>
+      </c>
+      <c r="B8" s="17">
+        <v>4</v>
+      </c>
+      <c r="C8" s="17">
+        <v>2</v>
+      </c>
+      <c r="D8" s="17">
+        <v>10</v>
+      </c>
+      <c r="E8" s="17">
+        <v>10</v>
+      </c>
+      <c r="F8" s="17">
+        <v>4</v>
+      </c>
+      <c r="G8" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="25" customHeight="1">
+      <c r="A9" s="17">
+        <v>8</v>
+      </c>
+      <c r="B9" s="17">
+        <v>2</v>
+      </c>
+      <c r="C9" s="17">
+        <v>1</v>
+      </c>
+      <c r="D9" s="17">
+        <v>3</v>
+      </c>
+      <c r="E9" s="17">
+        <v>6</v>
+      </c>
+      <c r="F9" s="17">
+        <v>4</v>
+      </c>
+      <c r="G9" s="17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="25" customHeight="1">
+      <c r="A10" s="17">
+        <v>9</v>
+      </c>
+      <c r="B10" s="17">
+        <v>1</v>
+      </c>
+      <c r="C10" s="17">
+        <v>1</v>
+      </c>
+      <c r="D10" s="17">
+        <v>1</v>
+      </c>
+      <c r="E10" s="17">
+        <v>1</v>
+      </c>
+      <c r="F10" s="17">
+        <v>4</v>
+      </c>
+      <c r="G10" s="17">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="I4:I7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="3" width="22" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1">
+      <c r="A2" s="17">
+        <v>0</v>
+      </c>
+      <c r="B2" s="17">
+        <v>15</v>
+      </c>
+      <c r="C2" s="17">
+        <v>0</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="25" customHeight="1">
+      <c r="A3" s="17">
+        <v>1</v>
+      </c>
+      <c r="B3" s="17">
+        <v>7</v>
+      </c>
+      <c r="C3" s="17">
+        <v>0</v>
+      </c>
+      <c r="E3" s="21"/>
+    </row>
+    <row r="4" spans="1:5" ht="25" customHeight="1">
+      <c r="A4" s="17">
+        <v>2</v>
+      </c>
+      <c r="B4" s="17">
+        <v>4</v>
+      </c>
+      <c r="C4" s="17">
+        <v>0</v>
+      </c>
+      <c r="E4" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="25" customHeight="1">
+      <c r="A5" s="17">
+        <v>3</v>
+      </c>
+      <c r="B5" s="17">
+        <v>3</v>
+      </c>
+      <c r="C5" s="17">
+        <v>1</v>
+      </c>
+      <c r="E5" s="21"/>
+    </row>
+    <row r="6" spans="1:5" ht="25" customHeight="1">
+      <c r="A6" s="17">
+        <v>4</v>
+      </c>
+      <c r="B6" s="17">
+        <v>2</v>
+      </c>
+      <c r="C6" s="17">
+        <v>1</v>
+      </c>
+      <c r="E6" s="21"/>
+    </row>
+    <row r="7" spans="1:5" ht="25" customHeight="1">
+      <c r="A7" s="17">
+        <v>5</v>
+      </c>
+      <c r="B7" s="17">
+        <v>1</v>
+      </c>
+      <c r="C7" s="17">
+        <v>1</v>
+      </c>
+      <c r="E7" s="21"/>
+    </row>
+    <row r="8" spans="1:5" ht="25" customHeight="1">
+      <c r="A8" s="17">
+        <v>6</v>
+      </c>
+      <c r="B8" s="17">
+        <v>1</v>
+      </c>
+      <c r="C8" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="25" customHeight="1">
+      <c r="A9" s="17">
+        <v>7</v>
+      </c>
+      <c r="B9" s="17">
+        <v>1</v>
+      </c>
+      <c r="C9" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="25" customHeight="1">
+      <c r="A10" s="17">
+        <v>8</v>
+      </c>
+      <c r="B10" s="17">
+        <v>1</v>
+      </c>
+      <c r="C10" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="25" customHeight="1">
+      <c r="A11" s="17">
+        <v>9</v>
+      </c>
+      <c r="B11" s="17">
+        <v>1</v>
+      </c>
+      <c r="C11" s="17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="25" customHeight="1">
+      <c r="A12" s="17">
+        <v>10</v>
+      </c>
+      <c r="B12" s="17">
+        <v>0</v>
+      </c>
+      <c r="C12" s="17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="25" customHeight="1">
+      <c r="A13" s="17">
+        <v>11</v>
+      </c>
+      <c r="B13" s="17">
+        <v>0</v>
+      </c>
+      <c r="C13" s="17">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="25" customHeight="1">
+      <c r="A14" s="17">
+        <v>12</v>
+      </c>
+      <c r="B14" s="17">
+        <v>0</v>
+      </c>
+      <c r="C14" s="17">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="E4:E7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="13.6"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="3" max="3" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="46.05" customHeight="1">
+      <c r="A1" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1" s="18" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="25" customHeight="1">
+      <c r="A2" s="17">
+        <v>12</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="25" customHeight="1">
+      <c r="A3" s="17">
+        <v>14</v>
+      </c>
+      <c r="C3" s="21"/>
+    </row>
+    <row r="4" spans="1:3" ht="25" customHeight="1">
+      <c r="A4" s="17">
+        <v>14</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="25" customHeight="1">
+      <c r="A5" s="17">
+        <v>18</v>
+      </c>
+      <c r="C5" s="21"/>
+    </row>
+    <row r="6" spans="1:3" ht="25" customHeight="1">
+      <c r="A6" s="17">
+        <v>21</v>
+      </c>
+      <c r="C6" s="21"/>
+    </row>
+    <row r="7" spans="1:3" ht="25" customHeight="1">
+      <c r="A7" s="17">
+        <v>23</v>
+      </c>
+      <c r="C7" s="21"/>
+    </row>
+    <row r="8" spans="1:3" ht="25" customHeight="1">
+      <c r="A8" s="17">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="25" customHeight="1">
+      <c r="A9" s="17">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="C4:C7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>